<commit_message>
Update model input variables for Uganda
</commit_message>
<xml_diff>
--- a/ssp_modeling/transformations/templates/calibrated/uganda/model_input_variables_uganda_se_calibrated.xlsx
+++ b/ssp_modeling/transformations/templates/calibrated/uganda/model_input_variables_uganda_se_calibrated.xlsx
@@ -618,85 +618,85 @@
         <v>46.50334192</v>
       </c>
       <c r="S2">
-        <v>56.53109005</v>
+        <v>53.89737328</v>
       </c>
       <c r="T2">
-        <v>68.72117165</v>
+        <v>62.46705563</v>
       </c>
       <c r="U2">
-        <v>83.5398615</v>
+        <v>72.39931747999999</v>
       </c>
       <c r="V2">
-        <v>101.5539795</v>
+        <v>83.91080896</v>
       </c>
       <c r="W2">
-        <v>123.4525719</v>
+        <v>97.25262758</v>
       </c>
       <c r="X2">
-        <v>150.0732673</v>
+        <v>112.7157954</v>
       </c>
       <c r="Y2">
-        <v>182.4343162</v>
+        <v>130.6376068</v>
       </c>
       <c r="Z2">
-        <v>199.2018542</v>
+        <v>140.0435145</v>
       </c>
       <c r="AA2">
-        <v>217.5104967</v>
+        <v>150.1266476</v>
       </c>
       <c r="AB2">
-        <v>237.5018864</v>
+        <v>160.9357662</v>
       </c>
       <c r="AC2">
-        <v>259.3306848</v>
+        <v>172.5231414</v>
       </c>
       <c r="AD2">
-        <v>283.165768</v>
+        <v>184.9448075</v>
       </c>
       <c r="AE2">
-        <v>321.6038221</v>
+        <v>199.3705025</v>
       </c>
       <c r="AF2">
-        <v>365.2596113</v>
+        <v>214.9214017</v>
       </c>
       <c r="AG2">
-        <v>414.841412</v>
+        <v>231.6852711</v>
       </c>
       <c r="AH2">
-        <v>471.1536446</v>
+        <v>249.7567222</v>
       </c>
       <c r="AI2">
-        <v>535.1099249</v>
+        <v>269.2377465</v>
       </c>
       <c r="AJ2">
-        <v>584.2918781</v>
+        <v>292.3921927</v>
       </c>
       <c r="AK2">
-        <v>637.9941446</v>
+        <v>317.5379213</v>
       </c>
       <c r="AL2">
-        <v>696.6321865</v>
+        <v>344.8461825</v>
       </c>
       <c r="AM2">
-        <v>760.6596507</v>
+        <v>374.5029542</v>
       </c>
       <c r="AN2">
-        <v>830.5718792</v>
+        <v>406.7102083</v>
       </c>
       <c r="AO2">
-        <v>912.1946695</v>
+        <v>443.314127</v>
       </c>
       <c r="AP2">
-        <v>1001.838776</v>
+        <v>483.2123985</v>
       </c>
       <c r="AQ2">
-        <v>1100.292478</v>
+        <v>526.7015143</v>
       </c>
       <c r="AR2">
-        <v>1208.421521</v>
+        <v>574.1046506</v>
       </c>
       <c r="AS2">
-        <v>1327.176729</v>
+        <v>625.7740692</v>
       </c>
     </row>
     <row r="3" spans="1:45">
@@ -957,112 +957,112 @@
         <v>1</v>
       </c>
       <c r="J5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="K5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="L5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="M5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="N5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="O5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="P5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="Q5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="R5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="S5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="T5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="U5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="V5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="W5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="X5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="Y5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="Z5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AA5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AB5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AC5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AD5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AE5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AF5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AG5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AH5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AI5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AJ5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AK5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AL5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AM5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AN5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AO5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AP5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AQ5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AR5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
       <c r="AS5">
-        <v>-0.1</v>
+        <v>-0.0865094146054103</v>
       </c>
     </row>
     <row r="6" spans="1:45">
@@ -1082,112 +1082,112 @@
         <v>1</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="K6">
-        <v>0.99</v>
+        <v>1.0395</v>
       </c>
       <c r="L6">
-        <v>0.98</v>
+        <v>1.029</v>
       </c>
       <c r="M6">
-        <v>0.97</v>
+        <v>1.0185</v>
       </c>
       <c r="N6">
-        <v>0.96</v>
+        <v>1.008</v>
       </c>
       <c r="O6">
-        <v>0.95</v>
+        <v>0.9975000000000001</v>
       </c>
       <c r="P6">
-        <v>0.9399999999999999</v>
+        <v>0.987</v>
       </c>
       <c r="Q6">
-        <v>0.93</v>
+        <v>0.9765</v>
       </c>
       <c r="R6">
-        <v>0.92</v>
+        <v>0.966</v>
       </c>
       <c r="S6">
-        <v>0.91</v>
+        <v>0.9555</v>
       </c>
       <c r="T6">
-        <v>0.9</v>
+        <v>0.945</v>
       </c>
       <c r="U6">
-        <v>0.89</v>
+        <v>0.9345</v>
       </c>
       <c r="V6">
-        <v>0.88</v>
+        <v>0.924</v>
       </c>
       <c r="W6">
-        <v>0.87</v>
+        <v>0.9135</v>
       </c>
       <c r="X6">
-        <v>0.86</v>
+        <v>0.903</v>
       </c>
       <c r="Y6">
-        <v>0.85</v>
+        <v>0.8925</v>
       </c>
       <c r="Z6">
-        <v>0.84</v>
+        <v>0.882</v>
       </c>
       <c r="AA6">
-        <v>0.83</v>
+        <v>0.8714999999999999</v>
       </c>
       <c r="AB6">
-        <v>0.82</v>
+        <v>0.861</v>
       </c>
       <c r="AC6">
-        <v>0.8100000000000001</v>
+        <v>0.8505000000000001</v>
       </c>
       <c r="AD6">
-        <v>0.8</v>
+        <v>0.8400000000000001</v>
       </c>
       <c r="AE6">
-        <v>0.79</v>
+        <v>0.8295000000000001</v>
       </c>
       <c r="AF6">
-        <v>0.78</v>
+        <v>0.8190000000000001</v>
       </c>
       <c r="AG6">
-        <v>0.77</v>
+        <v>0.8085000000000001</v>
       </c>
       <c r="AH6">
-        <v>0.76</v>
+        <v>0.798</v>
       </c>
       <c r="AI6">
-        <v>0.75</v>
+        <v>0.7875000000000001</v>
       </c>
       <c r="AJ6">
-        <v>0.74</v>
+        <v>0.777</v>
       </c>
       <c r="AK6">
-        <v>0.73</v>
+        <v>0.7665</v>
       </c>
       <c r="AL6">
-        <v>0.72</v>
+        <v>0.756</v>
       </c>
       <c r="AM6">
-        <v>0.71</v>
+        <v>0.7454999999999999</v>
       </c>
       <c r="AN6">
-        <v>0.7</v>
+        <v>0.735</v>
       </c>
       <c r="AO6">
-        <v>0.7</v>
+        <v>0.735</v>
       </c>
       <c r="AP6">
-        <v>0.7</v>
+        <v>0.735</v>
       </c>
       <c r="AQ6">
-        <v>0.7</v>
+        <v>0.735</v>
       </c>
       <c r="AR6">
-        <v>0.7</v>
+        <v>0.735</v>
       </c>
       <c r="AS6">
-        <v>0.7</v>
+        <v>0.735</v>
       </c>
     </row>
     <row r="7" spans="1:45">
@@ -1570,112 +1570,112 @@
         <v>1</v>
       </c>
       <c r="J10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="K10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="L10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="M10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="N10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="O10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="P10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="Q10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="R10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="S10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="T10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="U10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="V10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="W10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="X10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="Y10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="Z10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AA10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AB10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AC10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AD10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AE10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AF10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AG10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AH10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AI10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AJ10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AK10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AL10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AM10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AN10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AO10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AP10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AQ10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AR10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
       <c r="AS10">
-        <v>4.812222222</v>
+        <v>5.77288650882244</v>
       </c>
     </row>
     <row r="11" spans="1:45">

</xml_diff>